<commit_message>
docs(uat): drop CI/CD deploy line from Infra & Security sheet
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/UAT-Signoff.xlsx
+++ b/docs/uat/UAT-Signoff.xlsx
@@ -988,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1249,37 +1249,13 @@
       <c r="G11" s="11" t="inlineStr"/>
       <c r="H11" s="11" t="inlineStr"/>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Deploy pipeline</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Confirm a content/code change deploys to UAT.</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Push → CI → deploy works; revision healthy.</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A,Not tested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>